<commit_message>
refactor: split parser into modular parser files and add new folder operations and create all files inside that
</commit_message>
<xml_diff>
--- a/uploads/book1.xlsx
+++ b/uploads/book1.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>name</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>nd</t>
+  </si>
+  <si>
+    <t>bonus</t>
   </si>
 </sst>
 </file>
@@ -398,10 +401,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -411,8 +414,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -422,8 +428,11 @@
       <c r="C2">
         <v>454</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -433,8 +442,11 @@
       <c r="C3">
         <v>64</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -444,8 +456,11 @@
       <c r="C4">
         <v>2454</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -455,8 +470,11 @@
       <c r="C5">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -466,8 +484,11 @@
       <c r="C6">
         <v>78</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -477,8 +498,11 @@
       <c r="C7">
         <v>45</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -488,8 +512,11 @@
       <c r="C8">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -499,8 +526,11 @@
       <c r="C9">
         <v>44</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -510,8 +540,11 @@
       <c r="C10">
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -521,8 +554,11 @@
       <c r="C11">
         <v>487</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -532,8 +568,11 @@
       <c r="C12">
         <v>48</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -543,8 +582,11 @@
       <c r="C13">
         <v>322</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -554,8 +596,11 @@
       <c r="C14">
         <v>54</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -565,8 +610,11 @@
       <c r="C15">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -576,8 +624,11 @@
       <c r="C16">
         <v>12</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -587,8 +638,11 @@
       <c r="C17">
         <v>4644</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -598,8 +652,11 @@
       <c r="C18">
         <v>6494</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -609,8 +666,11 @@
       <c r="C19">
         <v>465</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -619,6 +679,9 @@
       </c>
       <c r="C20">
         <v>3145</v>
+      </c>
+      <c r="D20">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>